<commit_message>
Set starting and ending dates for kohteet according to changes in owners or habitants
</commit_message>
<xml_diff>
--- a/tests/data/test_data_import/DVV_update.xlsx
+++ b/tests/data/test_data_import/DVV_update.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="R1 rakennus" sheetId="1" state="visible" r:id="rId2"/>
@@ -2106,7 +2106,7 @@
         <v>62</v>
       </c>
       <c r="M8" s="2" t="n">
-        <v>20230201</v>
+        <v>20230117</v>
       </c>
       <c r="N8" s="2" t="n">
         <v>1</v>

</xml_diff>